<commit_message>
AI draft: mark least-sure pairs as review priority (kept, not removed); clarify checks are not linguistic evidence
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DPWV5aUdYeryeEaWbCPJ8f
</commit_message>
<xml_diff>
--- a/data/drafts/ai_draft_candidates.xlsx
+++ b/data/drafts/ai_draft_candidates.xlsx
@@ -59,7 +59,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="007F0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4B183"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -123,7 +128,13 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -491,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -553,22 +564,36 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>5. Rows marked PRIORITY are the ones the AI was least sure about. They are kept in the list and reviewed first; a reviewer may confirm or reject them like any other row. Nothing is pre-rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>6. Automated checks in this repository only confirm the written data is internally consistent (e.g. that two spellings differ by the intended Unicode change). They are NOT evidence that a pair is a genuine vowel-length or gemination contrast, or that the words are familiar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Design choices (not linguistic claims)</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="12" ht="70" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>36 vocab candidates: 6 'vowel length' pairs, 6 'gemination' pairs, 12 single words; 10 unknown-word (oov) candidates that must never be enrolled. No chillu letters are used on purpose, to avoid ZWJ encoding ambiguity. Romanisation is approximate, NOT IPA. Several candidates are phonetically close to one another (e.g. കളം/വളം, മല/മാല/മഴ); that is intended as a harder test but may not suit a first pilot.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="14" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="13" ht="14" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>This file cannot be loaded by review_sheet.py or the Sound2Word dataset tools by design.</t>
         </is>
@@ -585,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -597,9 +622,10 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
@@ -650,15 +676,20 @@
       </c>
       <c r="J1" s="5" t="inlineStr">
         <is>
+          <t>Review priority</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
           <t>AI concerns</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>Unknown-word closeness to enrolled (AI guess)</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -710,13 +741,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>Both very common. Check the long vowel is clearly longer in isolated speech.</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr"/>
-      <c r="L2" s="7" t="inlineStr">
+      <c r="L2" s="6" t="inlineStr"/>
+      <c r="M2" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -768,13 +804,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>Both very common. Check the long vowel is clearly longer in isolated speech.</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr"/>
-      <c r="L3" s="7" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -826,13 +867,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>'താരം' may be heard as 'star (celebrity)'; 'തരം' as 'kind, type, grade'. Confirm both are natural.</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr"/>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="L4" s="6" t="inlineStr"/>
+      <c r="M4" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -884,13 +930,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>'താരം' may be heard as 'star (celebrity)'; 'തരം' as 'kind, type, grade'. Confirm both are natural.</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr"/>
-      <c r="L5" s="7" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -942,13 +993,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Regional pronunciation of 'പടം' (picture/film) may vary.</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr"/>
-      <c r="L6" s="7" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr"/>
+      <c r="M6" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1000,13 +1056,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>Regional pronunciation of 'പടം' (picture/film) may vary.</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1058,13 +1119,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>Short words; confirm vowel length is the only audible difference.</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr"/>
-      <c r="L8" s="7" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr"/>
+      <c r="M8" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1116,13 +1182,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>Short words; confirm vowel length is the only audible difference.</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr"/>
-      <c r="L9" s="7" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1174,13 +1245,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>'നില' has several senses (floor, level, state); pick one context if needed.</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr"/>
-      <c r="L10" s="7" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr"/>
+      <c r="M10" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1232,13 +1308,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>'നില' has several senses (floor, level, state); pick one context if needed.</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr"/>
-      <c r="L11" s="7" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr"/>
+      <c r="M11" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1290,13 +1371,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>Short ൊ vs long ോ: confirm the contrast is length, not quality.</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr"/>
-      <c r="L12" s="7" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr"/>
+      <c r="M12" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1348,13 +1434,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Short ൊ vs long ോ: confirm the contrast is length, not quality.</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr"/>
-      <c r="L13" s="7" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr"/>
+      <c r="M13" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1406,13 +1497,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>Different parts of speech/semantic fields; confirm both familiar.</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr"/>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr"/>
+      <c r="M14" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1464,13 +1560,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>Different parts of speech/semantic fields; confirm both familiar.</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr"/>
-      <c r="L15" s="7" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr"/>
+      <c r="M15" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1522,13 +1623,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Close in sound to GP03 (കളം/വളം, കള്ളം/വള്ളം): useful hard negatives but may confuse a learner.</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr"/>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr"/>
+      <c r="M16" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1580,13 +1686,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>Close in sound to GP03 (കളം/വളം, കള്ളം/വള്ളം): useful hard negatives but may confuse a learner.</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="7" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr"/>
+      <c r="M17" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1638,13 +1749,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>Close in sound to GP02. 'വളം' = fertiliser (also other senses).</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr"/>
-      <c r="L18" s="7" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr"/>
+      <c r="M18" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1696,13 +1812,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>Close in sound to GP02. 'വളം' = fertiliser (also other senses).</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr"/>
-      <c r="L19" s="7" t="inlineStr">
+      <c r="L19" s="6" t="inlineStr"/>
+      <c r="M19" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1754,13 +1875,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Both extremely common.</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr"/>
-      <c r="L20" s="7" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr"/>
+      <c r="M20" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1812,13 +1938,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>Both extremely common.</t>
         </is>
       </c>
-      <c r="K21" s="6" t="inlineStr"/>
-      <c r="L21" s="7" t="inlineStr">
+      <c r="L21" s="6" t="inlineStr"/>
+      <c r="M21" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1870,13 +2001,18 @@
           <t>less sure</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>PRIORITY - confirm or reject</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
         <is>
           <t>'കട്ടി' has several senses (thickness, solid, lump); meaning may need fixing to one sense.</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr"/>
-      <c r="L22" s="7" t="inlineStr">
+      <c r="L22" s="6" t="inlineStr"/>
+      <c r="M22" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1928,13 +2064,18 @@
           <t>less sure</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>PRIORITY - confirm or reject</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>'കട്ടി' has several senses (thickness, solid, lump); meaning may need fixing to one sense.</t>
         </is>
       </c>
-      <c r="K23" s="6" t="inlineStr"/>
-      <c r="L23" s="7" t="inlineStr">
+      <c r="L23" s="6" t="inlineStr"/>
+      <c r="M23" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -1986,13 +2127,18 @@
           <t>less sure</t>
         </is>
       </c>
-      <c r="J24" s="6" t="inlineStr">
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>PRIORITY - confirm or reject</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>Is റ vs റ്റ a pure single/geminate contrast, or does quality also differ? Needs a phonetically aware reviewer.</t>
         </is>
       </c>
-      <c r="K24" s="6" t="inlineStr"/>
-      <c r="L24" s="7" t="inlineStr">
+      <c r="L24" s="6" t="inlineStr"/>
+      <c r="M24" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2044,13 +2190,18 @@
           <t>less sure</t>
         </is>
       </c>
-      <c r="J25" s="6" t="inlineStr">
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>PRIORITY - confirm or reject</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>Is റ vs റ്റ a pure single/geminate contrast, or does quality also differ? Needs a phonetically aware reviewer.</t>
         </is>
       </c>
-      <c r="K25" s="6" t="inlineStr"/>
-      <c r="L25" s="7" t="inlineStr">
+      <c r="L25" s="6" t="inlineStr"/>
+      <c r="M25" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2094,9 +2245,14 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J26" s="6" t="inlineStr"/>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
       <c r="K26" s="6" t="inlineStr"/>
-      <c r="L26" s="7" t="inlineStr">
+      <c r="L26" s="6" t="inlineStr"/>
+      <c r="M26" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2140,9 +2296,14 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J27" s="6" t="inlineStr"/>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
       <c r="K27" s="6" t="inlineStr"/>
-      <c r="L27" s="7" t="inlineStr">
+      <c r="L27" s="6" t="inlineStr"/>
+      <c r="M27" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2186,9 +2347,14 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J28" s="6" t="inlineStr"/>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
       <c r="K28" s="6" t="inlineStr"/>
-      <c r="L28" s="7" t="inlineStr">
+      <c r="L28" s="6" t="inlineStr"/>
+      <c r="M28" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2232,13 +2398,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J29" s="6" t="inlineStr">
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K29" s="6" t="inlineStr">
         <is>
           <t>Contains ഴ; shares it with പുഴ, പഴം (intentional spread, but similar endings).</t>
         </is>
       </c>
-      <c r="K29" s="6" t="inlineStr"/>
-      <c r="L29" s="7" t="inlineStr">
+      <c r="L29" s="6" t="inlineStr"/>
+      <c r="M29" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2282,13 +2453,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J30" s="6" t="inlineStr">
+      <c r="J30" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
         <is>
           <t>Shares ഴ with മഴ, പഴം.</t>
         </is>
       </c>
-      <c r="K30" s="6" t="inlineStr"/>
-      <c r="L30" s="7" t="inlineStr">
+      <c r="L30" s="6" t="inlineStr"/>
+      <c r="M30" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2332,13 +2508,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J31" s="6" t="inlineStr">
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>'banana' vs general 'fruit': pick the sense speakers use.</t>
         </is>
       </c>
-      <c r="K31" s="6" t="inlineStr"/>
-      <c r="L31" s="7" t="inlineStr">
+      <c r="L31" s="6" t="inlineStr"/>
+      <c r="M31" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2382,13 +2563,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J32" s="6" t="inlineStr">
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
         <is>
           <t>Geminate mm in a single word (no pair).</t>
         </is>
       </c>
-      <c r="K32" s="6" t="inlineStr"/>
-      <c r="L32" s="7" t="inlineStr">
+      <c r="L32" s="6" t="inlineStr"/>
+      <c r="M32" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2432,9 +2618,14 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J33" s="6" t="inlineStr"/>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
       <c r="K33" s="6" t="inlineStr"/>
-      <c r="L33" s="7" t="inlineStr">
+      <c r="L33" s="6" t="inlineStr"/>
+      <c r="M33" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2478,13 +2669,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J34" s="6" t="inlineStr">
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="inlineStr">
         <is>
           <t>Conjunct ങ്ങ: check spelling.</t>
         </is>
       </c>
-      <c r="K34" s="6" t="inlineStr"/>
-      <c r="L34" s="7" t="inlineStr">
+      <c r="L34" s="6" t="inlineStr"/>
+      <c r="M34" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2528,13 +2724,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J35" s="6" t="inlineStr">
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K35" s="6" t="inlineStr">
         <is>
           <t>Conjunct സ്ത: check spelling.</t>
         </is>
       </c>
-      <c r="K35" s="6" t="inlineStr"/>
-      <c r="L35" s="7" t="inlineStr">
+      <c r="L35" s="6" t="inlineStr"/>
+      <c r="M35" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2578,13 +2779,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J36" s="6" t="inlineStr">
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K36" s="6" t="inlineStr">
         <is>
           <t>Longer word (3 syllables) for length variety.</t>
         </is>
       </c>
-      <c r="K36" s="6" t="inlineStr"/>
-      <c r="L36" s="7" t="inlineStr">
+      <c r="L36" s="6" t="inlineStr"/>
+      <c r="M36" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2628,13 +2834,18 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J37" s="6" t="inlineStr">
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
         <is>
           <t>Long word (5 syllables); formal register.</t>
         </is>
       </c>
-      <c r="K37" s="6" t="inlineStr"/>
-      <c r="L37" s="7" t="inlineStr">
+      <c r="L37" s="6" t="inlineStr"/>
+      <c r="M37" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2678,17 +2889,22 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J38" s="6" t="inlineStr">
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
         <is>
           <t>Must NOT be enrolled; unknown-word test only.</t>
         </is>
       </c>
-      <c r="K38" s="6" t="inlineStr">
+      <c r="L38" s="6" t="inlineStr">
         <is>
           <t>far</t>
         </is>
       </c>
-      <c r="L38" s="7" t="inlineStr">
+      <c r="M38" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2732,17 +2948,22 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J39" s="6" t="inlineStr">
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K39" s="6" t="inlineStr">
         <is>
           <t>Must NOT be enrolled; unknown-word test only.</t>
         </is>
       </c>
-      <c r="K39" s="6" t="inlineStr">
+      <c r="L39" s="6" t="inlineStr">
         <is>
           <t>far</t>
         </is>
       </c>
-      <c r="L39" s="7" t="inlineStr">
+      <c r="M39" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2786,17 +3007,22 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J40" s="6" t="inlineStr">
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K40" s="6" t="inlineStr">
         <is>
           <t>Must NOT be enrolled; unknown-word test only.</t>
         </is>
       </c>
-      <c r="K40" s="6" t="inlineStr">
+      <c r="L40" s="6" t="inlineStr">
         <is>
           <t>far (one syllable)</t>
         </is>
       </c>
-      <c r="L40" s="7" t="inlineStr">
+      <c r="M40" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2840,17 +3066,22 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J41" s="6" t="inlineStr">
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="inlineStr">
         <is>
           <t>Must NOT be enrolled; unknown-word test only.</t>
         </is>
       </c>
-      <c r="K41" s="6" t="inlineStr">
+      <c r="L41" s="6" t="inlineStr">
         <is>
           <t>near (കട്ടി, കടി, പടി, പട്ടി)</t>
         </is>
       </c>
-      <c r="L41" s="7" t="inlineStr">
+      <c r="M41" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2894,17 +3125,22 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J42" s="6" t="inlineStr">
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K42" s="6" t="inlineStr">
         <is>
           <t>Must NOT be enrolled; unknown-word test only.</t>
         </is>
       </c>
-      <c r="K42" s="6" t="inlineStr">
+      <c r="L42" s="6" t="inlineStr">
         <is>
           <t>near (പഴം, മഴ, പുഴ share ഴ)</t>
         </is>
       </c>
-      <c r="L42" s="7" t="inlineStr">
+      <c r="M42" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -2948,17 +3184,22 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J43" s="6" t="inlineStr">
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K43" s="6" t="inlineStr">
         <is>
           <t>Must NOT be enrolled; unknown-word test only.</t>
         </is>
       </c>
-      <c r="K43" s="6" t="inlineStr">
+      <c r="L43" s="6" t="inlineStr">
         <is>
           <t>far</t>
         </is>
       </c>
-      <c r="L43" s="7" t="inlineStr">
+      <c r="M43" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -3002,17 +3243,22 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J44" s="6" t="inlineStr">
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K44" s="6" t="inlineStr">
         <is>
           <t>Must NOT be enrolled; unknown-word test only.</t>
         </is>
       </c>
-      <c r="K44" s="6" t="inlineStr">
+      <c r="L44" s="6" t="inlineStr">
         <is>
           <t>near (കുറി)</t>
         </is>
       </c>
-      <c r="L44" s="7" t="inlineStr">
+      <c r="M44" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -3056,17 +3302,22 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J45" s="6" t="inlineStr">
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K45" s="6" t="inlineStr">
         <is>
           <t>Must NOT be enrolled; unknown-word test only.</t>
         </is>
       </c>
-      <c r="K45" s="6" t="inlineStr">
+      <c r="L45" s="6" t="inlineStr">
         <is>
           <t>far</t>
         </is>
       </c>
-      <c r="L45" s="7" t="inlineStr">
+      <c r="M45" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -3110,17 +3361,22 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J46" s="6" t="inlineStr">
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K46" s="6" t="inlineStr">
         <is>
           <t>Must NOT be enrolled; unknown-word test only.</t>
         </is>
       </c>
-      <c r="K46" s="6" t="inlineStr">
+      <c r="L46" s="6" t="inlineStr">
         <is>
           <t>far (same meaning as താരം, unrelated sound)</t>
         </is>
       </c>
-      <c r="L46" s="7" t="inlineStr">
+      <c r="M46" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
@@ -3164,17 +3420,22 @@
           <t>more sure</t>
         </is>
       </c>
-      <c r="J47" s="6" t="inlineStr">
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="K47" s="6" t="inlineStr">
         <is>
           <t>Must NOT be enrolled; unknown-word test only.</t>
         </is>
       </c>
-      <c r="K47" s="6" t="inlineStr">
+      <c r="L47" s="6" t="inlineStr">
         <is>
           <t>far</t>
         </is>
       </c>
-      <c r="L47" s="7" t="inlineStr">
+      <c r="M47" s="8" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>

</xml_diff>